<commit_message>
Rename Suite planner to Dashboard
</commit_message>
<xml_diff>
--- a/artifacts/agent-customization/customized-budget.xlsx
+++ b/artifacts/agent-customization/customized-budget.xlsx
@@ -40,7 +40,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Category usage'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Category costs'!$A$1:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Monthly category summary'!$A$1:$H$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Profiles'!$A$1:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Profiles'!$A$1:$G$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Scenarios'!$A$1:$G$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Additional costs'!$A$1:$A$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Pricing'!$A$1:$R$3</definedName>
@@ -1738,7 +1738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1748,7 +1748,6 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1787,11 +1786,6 @@
           <t>cache_write_fraction</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>model_id</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1829,11 +1823,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Fixture A</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1871,7 +1860,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1909,10 +1897,9 @@
           <t>0</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H4"/>
+  <autoFilter ref="A1:G4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2559,7 +2546,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Schema 7; defaults 1</t>
+          <t>Schema 8; defaults 1</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4546,11 @@
       <c r="D2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Fixture A</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
@@ -4597,7 +4588,11 @@
       <c r="D3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Fixture A</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
@@ -4643,7 +4638,11 @@
       <c r="D4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Fixture A</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
@@ -4906,7 +4905,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>411aa4e8-9cb9-4909-8e5b-2179ec8724b8</t>
+          <t>9a30da2d-51e3-4595-8610-c3a3bcce101b</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5204,7 +5203,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>411aa4e8-9cb9-4909-8e5b-2179ec8724b8</t>
+          <t>9a30da2d-51e3-4595-8610-c3a3bcce101b</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -5455,7 +5454,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>28ea1562-0d88-4862-bfb7-8f5fe798d241</t>
+          <t>61996a9a-0f5e-4954-8b69-faac04d8be05</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -5465,7 +5464,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>411aa4e8-9cb9-4909-8e5b-2179ec8724b8</t>
+          <t>9a30da2d-51e3-4595-8610-c3a3bcce101b</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
@@ -5509,12 +5508,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>a9bfb02f-6024-4c37-8ace-07b95d1858d4</t>
+          <t>ef9ad5e2-11cc-48b8-bc67-1c2ef0ce96a1</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>411aa4e8-9cb9-4909-8e5b-2179ec8724b8</t>
+          <t>9a30da2d-51e3-4595-8610-c3a3bcce101b</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -5671,7 +5670,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>28ea1562-0d88-4862-bfb7-8f5fe798d241</t>
+          <t>61996a9a-0f5e-4954-8b69-faac04d8be05</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -5681,7 +5680,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>411aa4e8-9cb9-4909-8e5b-2179ec8724b8</t>
+          <t>9a30da2d-51e3-4595-8610-c3a3bcce101b</t>
         </is>
       </c>
       <c r="M8" s="2" t="n">
@@ -5725,12 +5724,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>a9bfb02f-6024-4c37-8ace-07b95d1858d4</t>
+          <t>ef9ad5e2-11cc-48b8-bc67-1c2ef0ce96a1</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>411aa4e8-9cb9-4909-8e5b-2179ec8724b8</t>
+          <t>9a30da2d-51e3-4595-8610-c3a3bcce101b</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -5887,7 +5886,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>28ea1562-0d88-4862-bfb7-8f5fe798d241</t>
+          <t>61996a9a-0f5e-4954-8b69-faac04d8be05</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -5897,7 +5896,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>411aa4e8-9cb9-4909-8e5b-2179ec8724b8</t>
+          <t>9a30da2d-51e3-4595-8610-c3a3bcce101b</t>
         </is>
       </c>
       <c r="M12" s="2" t="n">
@@ -5941,12 +5940,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>a9bfb02f-6024-4c37-8ace-07b95d1858d4</t>
+          <t>ef9ad5e2-11cc-48b8-bc67-1c2ef0ce96a1</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>411aa4e8-9cb9-4909-8e5b-2179ec8724b8</t>
+          <t>9a30da2d-51e3-4595-8610-c3a3bcce101b</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">

</xml_diff>